<commit_message>
many changes that are give after deployment
</commit_message>
<xml_diff>
--- a/docs/STAFF-DATA/015.xlsx
+++ b/docs/STAFF-DATA/015.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="28925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Velammal-Engineering-College-Backend\docs\STAFF-DATA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\VEC_Web_Engine\docs\STAFF-DATA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96AA9CE4-1A38-44E3-A88E-62CD268D1C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="80">
   <si>
     <t>Name</t>
   </si>
@@ -275,12 +274,15 @@
   </si>
   <si>
     <t>https://www.linkedin.com/in/sivatharani-boomiraja-54401b28b/</t>
+  </si>
+  <si>
+    <t>https://www.webofscience.com/wos/author/record/KGM-6216-2024</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -373,7 +375,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -397,6 +399,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -701,7 +706,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
@@ -711,11 +716,11 @@
     <col min="1" max="1" width="40.109375" style="6" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="29.44140625" style="6" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="21.88671875" customWidth="1"/>
-    <col min="6" max="6" width="28.44140625" style="6" customWidth="1"/>
-    <col min="7" max="7" width="20.33203125" customWidth="1"/>
-    <col min="8" max="8" width="3.5546875" style="6" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43" style="6" customWidth="1"/>
+    <col min="5" max="5" width="31.5546875" customWidth="1"/>
+    <col min="6" max="6" width="45" style="6" customWidth="1"/>
+    <col min="7" max="7" width="67.5546875" customWidth="1"/>
+    <col min="8" max="8" width="42.33203125" style="6" customWidth="1"/>
     <col min="9" max="9" width="31.44140625" style="6" customWidth="1"/>
     <col min="10" max="10" width="28.44140625" bestFit="1" customWidth="1"/>
   </cols>
@@ -901,6 +906,9 @@
       <c r="F7" s="4" t="s">
         <v>40</v>
       </c>
+      <c r="G7" s="9" t="s">
+        <v>79</v>
+      </c>
       <c r="H7" s="4" t="s">
         <v>41</v>
       </c>
@@ -1004,10 +1012,11 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{A5F98899-F30B-4293-B019-034FEA9638D3}"/>
-    <hyperlink ref="F3" r:id="rId2" xr:uid="{BF3A9B70-9AEA-4A70-B029-1A83F75D2D9D}"/>
-    <hyperlink ref="I4" r:id="rId3" xr:uid="{AA2C6452-0B04-4D63-8947-AC1B393FE427}"/>
-    <hyperlink ref="I10" r:id="rId4" xr:uid="{5573DF8A-7AFD-4543-8377-2314489BC0B3}"/>
+    <hyperlink ref="F2" r:id="rId1"/>
+    <hyperlink ref="F3" r:id="rId2"/>
+    <hyperlink ref="I4" r:id="rId3"/>
+    <hyperlink ref="I10" r:id="rId4"/>
+    <hyperlink ref="G7" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>